<commit_message>
fix: 统一 T004/T005 虎力值奖励(10/15->15/10) 与 PRD 2.4/2.5 对齐
</commit_message>
<xml_diff>
--- a/泰小虎任务完成条件配置PRD v2.2.xlsx
+++ b/泰小虎任务完成条件配置PRD v2.2.xlsx
@@ -1201,6 +1201,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="16.5" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
         <is>
@@ -1357,10 +1358,8 @@
           <t>dialogue_send（is_first_message==true）</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="E8" t="n">
+        <v>15</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -1389,14 +1388,12 @@
           <t>recommend_view（recommend_source==service）</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
+      <c r="E9" t="n">
+        <v>10</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>复用·事件有效（缺 service 枚举）</t>
+          <t>复用·事件有效（service 枚举已补）</t>
         </is>
       </c>
     </row>
@@ -3757,6 +3754,7 @@
       <c r="P1" s="2" t="n"/>
       <c r="Q1" s="2" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -3928,10 +3926,8 @@
           <t>is_first_message == true（本次对话首条消息）</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="D16" s="6" t="n">
+        <v>15</v>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
@@ -4444,6 +4440,7 @@
       <c r="P1" s="2" t="n"/>
       <c r="Q1" s="2" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -4615,10 +4612,8 @@
           <t>recommend_source == service（健康好物 Tab 曝光）</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
+      <c r="D16" s="6" t="n">
+        <v>10</v>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>

</xml_diff>